<commit_message>
Added Exercise 4A docs
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -8,15 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charlespalacios\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{576770BD-610F-467E-B1C0-9F5EC9BD2B59}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{AEE46466-96E4-44A4-9CBC-934D4ED94158}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{5216206F-9075-4552-B206-7893CFD4434E}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{FC12ADFC-1BA8-4B32-B226-434D0D04D022}"/>
   </bookViews>
   <sheets>
     <sheet name="GTrends_milkshake_hamburger_202" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">GTrends_milkshake_hamburger_202!$A$1:$E$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">GTrends_milkshake_hamburger_202!$A$1:$E$52</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -44,166 +44,166 @@
     <t>Region</t>
   </si>
   <si>
-    <t>Milkshake: (4/9/25 - 4/9/26)</t>
-  </si>
-  <si>
-    <t>Hamburger: (4/9/25 - 4/9/26)</t>
-  </si>
-  <si>
-    <t>Breakup: (4/9/25 - 4/9/26)</t>
+    <t>Milkshake: (2/1/24 - 2/28/25)</t>
+  </si>
+  <si>
+    <t>Hamburger: (2/1/24 - 2/28/25)</t>
+  </si>
+  <si>
+    <t>Breakup: (2/1/24 - 2/28/25)</t>
+  </si>
+  <si>
+    <t>North Carolina</t>
+  </si>
+  <si>
+    <t>South Carolina</t>
+  </si>
+  <si>
+    <t>Kentucky</t>
   </si>
   <si>
     <t>Alabama</t>
   </si>
   <si>
-    <t>North Carolina</t>
-  </si>
-  <si>
-    <t>Kentucky</t>
+    <t>Arizona</t>
   </si>
   <si>
     <t>Tennessee</t>
   </si>
   <si>
-    <t>South Carolina</t>
-  </si>
-  <si>
     <t>Utah</t>
   </si>
   <si>
+    <t>Illinois</t>
+  </si>
+  <si>
+    <t>Oklahoma</t>
+  </si>
+  <si>
+    <t>Indiana</t>
+  </si>
+  <si>
+    <t>Georgia</t>
+  </si>
+  <si>
+    <t>Virginia</t>
+  </si>
+  <si>
+    <t>Arkansas</t>
+  </si>
+  <si>
     <t>Ohio</t>
   </si>
   <si>
+    <t>Connecticut</t>
+  </si>
+  <si>
+    <t>Delaware</t>
+  </si>
+  <si>
+    <t>Mississippi</t>
+  </si>
+  <si>
     <t>West Virginia</t>
   </si>
   <si>
-    <t>Oklahoma</t>
+    <t>Florida</t>
+  </si>
+  <si>
+    <t>Nevada</t>
+  </si>
+  <si>
+    <t>Maryland</t>
+  </si>
+  <si>
+    <t>Rhode Island</t>
+  </si>
+  <si>
+    <t>Kansas</t>
+  </si>
+  <si>
+    <t>Pennsylvania</t>
+  </si>
+  <si>
+    <t>Texas</t>
   </si>
   <si>
     <t>Missouri</t>
   </si>
   <si>
-    <t>Virginia</t>
-  </si>
-  <si>
-    <t>Delaware</t>
-  </si>
-  <si>
-    <t>Arkansas</t>
-  </si>
-  <si>
-    <t>Illinois</t>
-  </si>
-  <si>
-    <t>Georgia</t>
-  </si>
-  <si>
-    <t>Indiana</t>
-  </si>
-  <si>
-    <t>Mississippi</t>
-  </si>
-  <si>
-    <t>Nevada</t>
-  </si>
-  <si>
-    <t>Florida</t>
+    <t>Michigan</t>
+  </si>
+  <si>
+    <t>Wisconsin</t>
+  </si>
+  <si>
+    <t>California</t>
   </si>
   <si>
     <t>New Jersey</t>
   </si>
   <si>
-    <t>Texas</t>
-  </si>
-  <si>
-    <t>Pennsylvania</t>
+    <t>Washington</t>
+  </si>
+  <si>
+    <t>Idaho</t>
+  </si>
+  <si>
+    <t>Louisiana</t>
+  </si>
+  <si>
+    <t>Iowa</t>
+  </si>
+  <si>
+    <t>North Dakota</t>
+  </si>
+  <si>
+    <t>Minnesota</t>
+  </si>
+  <si>
+    <t>New Hampshire</t>
   </si>
   <si>
     <t>Colorado</t>
   </si>
   <si>
-    <t>Arizona</t>
-  </si>
-  <si>
-    <t>Maryland</t>
-  </si>
-  <si>
-    <t>Louisiana</t>
-  </si>
-  <si>
-    <t>Idaho</t>
-  </si>
-  <si>
-    <t>Kansas</t>
-  </si>
-  <si>
-    <t>California</t>
-  </si>
-  <si>
-    <t>Rhode Island</t>
-  </si>
-  <si>
     <t>Oregon</t>
   </si>
   <si>
+    <t>Nebraska</t>
+  </si>
+  <si>
+    <t>Massachusetts</t>
+  </si>
+  <si>
+    <t>New York</t>
+  </si>
+  <si>
+    <t>South Dakota</t>
+  </si>
+  <si>
     <t>New Mexico</t>
   </si>
   <si>
-    <t>Iowa</t>
-  </si>
-  <si>
-    <t>Wisconsin</t>
-  </si>
-  <si>
-    <t>Michigan</t>
-  </si>
-  <si>
-    <t>Minnesota</t>
-  </si>
-  <si>
-    <t>North Dakota</t>
-  </si>
-  <si>
-    <t>Nebraska</t>
-  </si>
-  <si>
     <t>Wyoming</t>
   </si>
   <si>
-    <t>Connecticut</t>
-  </si>
-  <si>
-    <t>Washington</t>
-  </si>
-  <si>
-    <t>New York</t>
-  </si>
-  <si>
-    <t>Massachusetts</t>
-  </si>
-  <si>
-    <t>New Hampshire</t>
-  </si>
-  <si>
     <t>Maine</t>
   </si>
   <si>
+    <t>Montana</t>
+  </si>
+  <si>
+    <t>Vermont</t>
+  </si>
+  <si>
+    <t>Hawaii</t>
+  </si>
+  <si>
     <t>Alaska</t>
   </si>
   <si>
-    <t>Hawaii</t>
-  </si>
-  <si>
-    <t>South Dakota</t>
-  </si>
-  <si>
-    <t>Montana</t>
-  </si>
-  <si>
     <t>District of Columbia</t>
-  </si>
-  <si>
-    <t>Vermont</t>
   </si>
   <si>
     <t># of Regions</t>
@@ -696,7 +696,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="1" fillId="23" borderId="0" xfId="32"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="0" xfId="31"/>
   </cellXfs>
   <cellStyles count="42">
     <cellStyle name="20% - Accent1" xfId="19" builtinId="30" customBuiltin="1"/>
@@ -1071,15 +1071,16 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A484486-48AF-4B79-AD88-9C86AD6007DA}">
+<worksheet xmlns="http://purl.oclc.org/ooxml/spreadsheetml/main" xmlns:r="http://purl.oclc.org/ooxml/officeDocument/relationships" xmlns:v="urn:schemas-microsoft-com:vml" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C1D0EC21-D836-45DE-831B-814566909D27}">
   <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="10.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16.77734375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="25.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="24.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="26.5546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="25.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.5546875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1103,7 +1104,7 @@
         <v>55</v>
       </c>
       <c r="H1" s="2">
-        <f>COUNTA(B2:B52)</f>
+        <f>COUNTA(D2:D52)</f>
         <v>51</v>
       </c>
     </row>
@@ -1118,10 +1119,10 @@
         <v>0.63</v>
       </c>
       <c r="D2" s="1">
-        <v>0.23</v>
+        <v>0.24</v>
       </c>
       <c r="E2" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
@@ -1129,16 +1130,16 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>49</v>
+        <v>5</v>
       </c>
       <c r="C3" s="1">
-        <v>0.7</v>
+        <v>0.68</v>
       </c>
       <c r="D3" s="1">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="E3" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
@@ -1146,16 +1147,16 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="C4" s="1">
-        <v>0.65</v>
+        <v>0.63</v>
       </c>
       <c r="D4" s="1">
-        <v>0.2</v>
+        <v>0.24</v>
       </c>
       <c r="E4" s="1">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
@@ -1163,16 +1164,16 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>16</v>
+        <v>7</v>
       </c>
       <c r="C5" s="1">
-        <v>0.65</v>
+        <v>0.64</v>
       </c>
       <c r="D5" s="1">
-        <v>0.22</v>
+        <v>0.24</v>
       </c>
       <c r="E5" s="1">
-        <v>0.13</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
@@ -1180,16 +1181,16 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>32</v>
+        <v>8</v>
       </c>
       <c r="C6" s="1">
-        <v>0.62</v>
+        <v>0.64</v>
       </c>
       <c r="D6" s="1">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="E6" s="1">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -1197,16 +1198,16 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="C7" s="1">
-        <v>0.64</v>
+        <v>0.66</v>
       </c>
       <c r="D7" s="1">
-        <v>0.2</v>
+        <v>0.21</v>
       </c>
       <c r="E7" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -1214,16 +1215,16 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>43</v>
+        <v>10</v>
       </c>
       <c r="C8" s="1">
-        <v>0.63</v>
+        <v>0.66</v>
       </c>
       <c r="D8" s="1">
         <v>0.21</v>
       </c>
       <c r="E8" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
@@ -1231,16 +1232,16 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="C9" s="1">
-        <v>0.62</v>
+        <v>0.61</v>
       </c>
       <c r="D9" s="1">
         <v>0.24</v>
       </c>
       <c r="E9" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
@@ -1248,16 +1249,16 @@
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>12</v>
       </c>
       <c r="C10" s="1">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="D10" s="1">
-        <v>0.17</v>
+        <v>0.2</v>
       </c>
       <c r="E10" s="1">
-        <v>0.19</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
@@ -1265,7 +1266,7 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="C11" s="1">
         <v>0.63</v>
@@ -1282,7 +1283,7 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="C12" s="1">
         <v>0.62</v>
@@ -1299,16 +1300,16 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>50</v>
+        <v>15</v>
       </c>
       <c r="C13" s="1">
-        <v>0.68</v>
+        <v>0.61</v>
       </c>
       <c r="D13" s="1">
+        <v>0.24</v>
+      </c>
+      <c r="E13" s="1">
         <v>0.15</v>
-      </c>
-      <c r="E13" s="1">
-        <v>0.17</v>
       </c>
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.3">
@@ -1316,13 +1317,13 @@
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>30</v>
+        <v>16</v>
       </c>
       <c r="C14" s="1">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="D14" s="1">
-        <v>0.19</v>
+        <v>0.21</v>
       </c>
       <c r="E14" s="1">
         <v>0.13</v>
@@ -1336,13 +1337,13 @@
         <v>17</v>
       </c>
       <c r="C15" s="1">
-        <v>0.62</v>
+        <v>0.65</v>
       </c>
       <c r="D15" s="1">
         <v>0.22</v>
       </c>
       <c r="E15" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
@@ -1350,16 +1351,16 @@
         <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C16" s="1">
-        <v>0.64</v>
+        <v>0.63</v>
       </c>
       <c r="D16" s="1">
         <v>0.22</v>
       </c>
       <c r="E16" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
@@ -1367,16 +1368,16 @@
         <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>36</v>
+        <v>19</v>
       </c>
       <c r="C17" s="1">
-        <v>0.67</v>
+        <v>0.64</v>
       </c>
       <c r="D17" s="1">
-        <v>0.19</v>
+        <v>0.23</v>
       </c>
       <c r="E17" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -1384,16 +1385,16 @@
         <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="C18" s="1">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D18" s="1">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="E18" s="1">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
@@ -1401,7 +1402,7 @@
         <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="C19" s="1">
         <v>0.64</v>
@@ -1418,16 +1419,16 @@
         <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>29</v>
+        <v>22</v>
       </c>
       <c r="C20" s="1">
         <v>0.63</v>
       </c>
       <c r="D20" s="1">
-        <v>0.21</v>
+        <v>0.23</v>
       </c>
       <c r="E20" s="1">
-        <v>0.16</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
@@ -1435,16 +1436,16 @@
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>48</v>
+        <v>23</v>
       </c>
       <c r="C21" s="1">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="D21" s="1">
-        <v>0.18</v>
+        <v>0.2</v>
       </c>
       <c r="E21" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
@@ -1452,16 +1453,16 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C22" s="1">
-        <v>0.6</v>
+        <v>0.62</v>
       </c>
       <c r="D22" s="1">
         <v>0.23</v>
       </c>
       <c r="E22" s="1">
-        <v>0.17</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1469,16 +1470,16 @@
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="C23" s="1">
-        <v>0.61</v>
+        <v>0.64</v>
       </c>
       <c r="D23" s="1">
-        <v>0.2</v>
+        <v>0.23</v>
       </c>
       <c r="E23" s="1">
-        <v>0.19</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1486,16 +1487,16 @@
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="C24" s="1">
-        <v>0.67</v>
+        <v>0.68</v>
       </c>
       <c r="D24" s="1">
         <v>0.19</v>
       </c>
       <c r="E24" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1503,13 +1504,13 @@
         <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="C25" s="1">
-        <v>0.66</v>
+        <v>0.63</v>
       </c>
       <c r="D25" s="1">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="E25" s="1">
         <v>0.15</v>
@@ -1520,13 +1521,13 @@
         <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="C26" s="1">
-        <v>0.65</v>
+        <v>0.67</v>
       </c>
       <c r="D26" s="1">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="E26" s="1">
         <v>0.13</v>
@@ -1537,16 +1538,16 @@
         <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C27" s="1">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="D27" s="1">
-        <v>0.22</v>
+        <v>0.2</v>
       </c>
       <c r="E27" s="1">
-        <v>0.13</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1554,16 +1555,16 @@
         <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>52</v>
+        <v>30</v>
       </c>
       <c r="C28" s="1">
-        <v>0.73</v>
+        <v>0.67</v>
       </c>
       <c r="D28" s="1">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="E28" s="1">
-        <v>0.12</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
@@ -1571,16 +1572,16 @@
         <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>41</v>
+        <v>31</v>
       </c>
       <c r="C29" s="1">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="D29" s="1">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="E29" s="1">
-        <v>0.13</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1588,13 +1589,13 @@
         <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>21</v>
+        <v>32</v>
       </c>
       <c r="C30" s="1">
-        <v>0.65</v>
+        <v>0.66</v>
       </c>
       <c r="D30" s="1">
-        <v>0.2</v>
+        <v>0.19</v>
       </c>
       <c r="E30" s="1">
         <v>0.15</v>
@@ -1605,16 +1606,16 @@
         <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>47</v>
+        <v>33</v>
       </c>
       <c r="C31" s="1">
-        <v>0.67</v>
+        <v>0.61</v>
       </c>
       <c r="D31" s="1">
-        <v>0.19</v>
+        <v>0.22</v>
       </c>
       <c r="E31" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.17</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
@@ -1622,16 +1623,16 @@
         <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="C32" s="1">
-        <v>0.59</v>
+        <v>0.67</v>
       </c>
       <c r="D32" s="1">
-        <v>0.23</v>
+        <v>0.19</v>
       </c>
       <c r="E32" s="1">
-        <v>0.18</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1642,13 +1643,13 @@
         <v>35</v>
       </c>
       <c r="C33" s="1">
-        <v>0.64</v>
+        <v>0.69</v>
       </c>
       <c r="D33" s="1">
-        <v>0.21</v>
+        <v>0.18</v>
       </c>
       <c r="E33" s="1">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1656,16 +1657,16 @@
         <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="C34" s="1">
-        <v>0.6</v>
+        <v>0.68</v>
       </c>
       <c r="D34" s="1">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="E34" s="1">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -1673,16 +1674,16 @@
         <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>5</v>
+        <v>37</v>
       </c>
       <c r="C35" s="1">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="D35" s="1">
-        <v>0.23</v>
+        <v>0.19</v>
       </c>
       <c r="E35" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
@@ -1690,13 +1691,13 @@
         <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="C36" s="1">
-        <v>0.69</v>
+        <v>0.7</v>
       </c>
       <c r="D36" s="1">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="E36" s="1">
         <v>0.12</v>
@@ -1707,16 +1708,16 @@
         <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>10</v>
+        <v>39</v>
       </c>
       <c r="C37" s="1">
-        <v>0.63</v>
+        <v>0.68</v>
       </c>
       <c r="D37" s="1">
-        <v>0.22</v>
+        <v>0.18</v>
       </c>
       <c r="E37" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
@@ -1724,13 +1725,13 @@
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="C38" s="1">
-        <v>0.68</v>
+        <v>0.67</v>
       </c>
       <c r="D38" s="1">
-        <v>0.19</v>
+        <v>0.2</v>
       </c>
       <c r="E38" s="1">
         <v>0.13</v>
@@ -1741,16 +1742,16 @@
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="C39" s="1">
-        <v>0.66</v>
+        <v>0.68</v>
       </c>
       <c r="D39" s="1">
-        <v>0.19</v>
+        <v>0.18</v>
       </c>
       <c r="E39" s="1">
-        <v>0.15</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1758,16 +1759,16 @@
         <v>39</v>
       </c>
       <c r="B40" t="s">
-        <v>25</v>
+        <v>42</v>
       </c>
       <c r="C40" s="1">
-        <v>0.6</v>
+        <v>0.69</v>
       </c>
       <c r="D40" s="1">
-        <v>0.22</v>
+        <v>0.18</v>
       </c>
       <c r="E40" s="1">
-        <v>0.18</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1775,16 +1776,16 @@
         <v>40</v>
       </c>
       <c r="B41" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="C41" s="1">
-        <v>0.62</v>
+        <v>0.68</v>
       </c>
       <c r="D41" s="1">
-        <v>0.22</v>
+        <v>0.19</v>
       </c>
       <c r="E41" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -1792,16 +1793,16 @@
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>8</v>
+        <v>44</v>
       </c>
       <c r="C42" s="1">
         <v>0.63</v>
       </c>
       <c r="D42" s="1">
-        <v>0.24</v>
+        <v>0.21</v>
       </c>
       <c r="E42" s="1">
-        <v>0.13</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1809,16 +1810,16 @@
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>51</v>
+        <v>45</v>
       </c>
       <c r="C43" s="1">
-        <v>0.76</v>
+        <v>0.64</v>
       </c>
       <c r="D43" s="1">
-        <v>0.13</v>
+        <v>0.2</v>
       </c>
       <c r="E43" s="1">
-        <v>0.11</v>
+        <v>0.16</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1826,16 +1827,16 @@
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>7</v>
+        <v>46</v>
       </c>
       <c r="C44" s="1">
-        <v>0.62</v>
+        <v>0.75</v>
       </c>
       <c r="D44" s="1">
-        <v>0.22</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E44" s="1">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
@@ -1843,16 +1844,16 @@
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="C45" s="1">
-        <v>0.64</v>
+        <v>0.68</v>
       </c>
       <c r="D45" s="1">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="E45" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.15</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -1860,16 +1861,16 @@
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>9</v>
+        <v>48</v>
       </c>
       <c r="C46" s="1">
-        <v>0.64</v>
+        <v>0.7</v>
       </c>
       <c r="D46" s="1">
-        <v>0.22</v>
+        <v>0.17</v>
       </c>
       <c r="E46" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
@@ -1877,16 +1878,16 @@
         <v>46</v>
       </c>
       <c r="B47" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C47" s="1">
         <v>0.69</v>
       </c>
       <c r="D47" s="1">
-        <v>0.15</v>
+        <v>0.18</v>
       </c>
       <c r="E47" s="1">
-        <v>0.16</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -1894,16 +1895,16 @@
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>14</v>
+        <v>50</v>
       </c>
       <c r="C48" s="1">
-        <v>0.63</v>
+        <v>0.75</v>
       </c>
       <c r="D48" s="1">
-        <v>0.22</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="E48" s="1">
-        <v>0.15</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
@@ -1911,16 +1912,16 @@
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>44</v>
+        <v>51</v>
       </c>
       <c r="C49" s="1">
-        <v>0.66</v>
+        <v>0.69</v>
       </c>
       <c r="D49" s="1">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="E49" s="1">
-        <v>0.16</v>
+        <v>0.14000000000000001</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -1928,16 +1929,16 @@
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>11</v>
+        <v>52</v>
       </c>
       <c r="C50" s="1">
-        <v>0.63</v>
+        <v>0.72</v>
       </c>
       <c r="D50" s="1">
-        <v>0.22</v>
+        <v>0.15</v>
       </c>
       <c r="E50" s="1">
-        <v>0.15</v>
+        <v>0.13</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
@@ -1945,13 +1946,13 @@
         <v>50</v>
       </c>
       <c r="B51" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="C51" s="1">
-        <v>0.68</v>
+        <v>0.71</v>
       </c>
       <c r="D51" s="1">
-        <v>0.18</v>
+        <v>0.15</v>
       </c>
       <c r="E51" s="1">
         <v>0.14000000000000001</v>
@@ -1962,20 +1963,20 @@
         <v>51</v>
       </c>
       <c r="B52" t="s">
-        <v>42</v>
+        <v>54</v>
       </c>
       <c r="C52" s="1">
-        <v>0.68</v>
+        <v>0.66</v>
       </c>
       <c r="D52" s="1">
-        <v>0.18</v>
+        <v>0.17</v>
       </c>
       <c r="E52" s="1">
-        <v>0.14000000000000001</v>
+        <v>0.17</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:E53" xr:uid="{7A484486-48AF-4B79-AD88-9C86AD6007DA}"/>
+  <autoFilter ref="A1:E52" xr:uid="{C1D0EC21-D836-45DE-831B-814566909D27}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>